<commit_message>
Added master data and updated course combination
</commit_message>
<xml_diff>
--- a/COURSE COMBINATION.xlsx
+++ b/COURSE COMBINATION.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prith\Documents\AI_Projects\MACE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7589BAF-C925-4F5B-B494-54F4AFB2412E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2235A8E7-5A36-4C0A-8EAA-ABDBAD4B003B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -775,34 +775,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -812,9 +791,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -823,6 +799,30 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1326,31 +1326,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2"/>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
     </row>
     <row r="4" spans="1:5" ht="16">
       <c r="A4" s="3" t="s">
@@ -1368,7 +1368,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="16">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="44" t="s">
         <v>94</v>
       </c>
       <c r="B5" s="6"/>
@@ -1383,7 +1383,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="16">
-      <c r="A6" s="53"/>
+      <c r="A6" s="45"/>
       <c r="B6" s="10"/>
       <c r="C6" s="11">
         <v>3102</v>
@@ -1396,7 +1396,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="16">
-      <c r="A7" s="53"/>
+      <c r="A7" s="45"/>
       <c r="B7" s="10"/>
       <c r="C7" s="7">
         <v>3103</v>
@@ -1409,7 +1409,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="16">
-      <c r="A8" s="53"/>
+      <c r="A8" s="45"/>
       <c r="B8" s="10"/>
       <c r="C8" s="11">
         <v>3104</v>
@@ -1422,7 +1422,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="16">
-      <c r="A9" s="53"/>
+      <c r="A9" s="45"/>
       <c r="B9" s="10"/>
       <c r="C9" s="11">
         <v>3105</v>
@@ -1435,7 +1435,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="16">
-      <c r="A10" s="53"/>
+      <c r="A10" s="45"/>
       <c r="B10" s="10"/>
       <c r="C10" s="11">
         <v>3106</v>
@@ -1448,7 +1448,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="16">
-      <c r="A11" s="53"/>
+      <c r="A11" s="45"/>
       <c r="B11" s="10"/>
       <c r="C11" s="11">
         <v>3107</v>
@@ -1461,7 +1461,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="16">
-      <c r="A12" s="53"/>
+      <c r="A12" s="45"/>
       <c r="B12" s="10"/>
       <c r="C12" s="11">
         <v>3108</v>
@@ -1469,12 +1469,12 @@
       <c r="D12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="44" t="s">
+      <c r="E12" s="36" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16">
-      <c r="A13" s="53"/>
+      <c r="A13" s="45"/>
       <c r="B13" s="10"/>
       <c r="C13" s="12">
         <v>3109</v>
@@ -1487,16 +1487,16 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="53"/>
-      <c r="B14" s="37" t="s">
+      <c r="A14" s="45"/>
+      <c r="B14" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
     </row>
     <row r="15" spans="1:5" ht="16">
-      <c r="A15" s="53"/>
+      <c r="A15" s="45"/>
       <c r="B15" s="10"/>
       <c r="C15" s="14" t="s">
         <v>3</v>
@@ -1509,7 +1509,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="16">
-      <c r="A16" s="53"/>
+      <c r="A16" s="45"/>
       <c r="B16" s="10"/>
       <c r="C16" s="16">
         <v>3201</v>
@@ -1522,7 +1522,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="16">
-      <c r="A17" s="53"/>
+      <c r="A17" s="45"/>
       <c r="B17" s="10"/>
       <c r="C17" s="16">
         <v>3202</v>
@@ -1535,8 +1535,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="16">
-      <c r="A18" s="53"/>
-      <c r="B18" s="51" t="s">
+      <c r="A18" s="45"/>
+      <c r="B18" s="40" t="s">
         <v>95</v>
       </c>
       <c r="C18" s="16">
@@ -1550,7 +1550,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="16">
-      <c r="A19" s="53"/>
+      <c r="A19" s="45"/>
       <c r="B19" s="10"/>
       <c r="C19" s="11">
         <v>3204</v>
@@ -1563,7 +1563,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="16">
-      <c r="A20" s="53"/>
+      <c r="A20" s="45"/>
       <c r="B20" s="10"/>
       <c r="C20" s="11">
         <v>3205</v>
@@ -1576,7 +1576,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="16">
-      <c r="A21" s="53"/>
+      <c r="A21" s="45"/>
       <c r="B21" s="10"/>
       <c r="C21" s="11">
         <v>3206</v>
@@ -1589,7 +1589,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="16">
-      <c r="A22" s="53"/>
+      <c r="A22" s="45"/>
       <c r="B22" s="10"/>
       <c r="C22" s="11">
         <v>3207</v>
@@ -1602,7 +1602,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="16">
-      <c r="A23" s="53"/>
+      <c r="A23" s="45"/>
       <c r="B23" s="10"/>
       <c r="C23" s="11">
         <v>3208</v>
@@ -1610,12 +1610,12 @@
       <c r="D23" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="36" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="16">
-      <c r="A24" s="53"/>
+      <c r="A24" s="45"/>
       <c r="B24" s="10"/>
       <c r="C24" s="11">
         <v>3209</v>
@@ -1628,7 +1628,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="16">
-      <c r="A25" s="53"/>
+      <c r="A25" s="45"/>
       <c r="B25" s="10"/>
       <c r="C25" s="12">
         <v>3210</v>
@@ -1641,16 +1641,16 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="53"/>
-      <c r="B26" s="37" t="s">
+      <c r="A26" s="45"/>
+      <c r="B26" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
     </row>
     <row r="27" spans="1:5" ht="16">
-      <c r="A27" s="53"/>
+      <c r="A27" s="45"/>
       <c r="B27" s="10"/>
       <c r="C27" s="14" t="s">
         <v>3</v>
@@ -1663,7 +1663,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="16">
-      <c r="A28" s="53"/>
+      <c r="A28" s="45"/>
       <c r="B28" s="10"/>
       <c r="C28" s="16">
         <v>3301</v>
@@ -1676,7 +1676,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="16">
-      <c r="A29" s="53"/>
+      <c r="A29" s="45"/>
       <c r="B29" s="10"/>
       <c r="C29" s="16">
         <v>3302</v>
@@ -1689,7 +1689,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="16">
-      <c r="A30" s="53"/>
+      <c r="A30" s="45"/>
       <c r="B30" s="10"/>
       <c r="C30" s="16">
         <v>3303</v>
@@ -1702,7 +1702,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="16">
-      <c r="A31" s="53"/>
+      <c r="A31" s="45"/>
       <c r="B31" s="10"/>
       <c r="C31" s="16">
         <v>3304</v>
@@ -1715,7 +1715,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="16">
-      <c r="A32" s="53"/>
+      <c r="A32" s="45"/>
       <c r="B32" s="10"/>
       <c r="C32" s="16">
         <v>3305</v>
@@ -1728,7 +1728,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="16">
-      <c r="A33" s="53"/>
+      <c r="A33" s="45"/>
       <c r="B33" s="10"/>
       <c r="C33" s="16">
         <v>3306</v>
@@ -1741,7 +1741,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="16">
-      <c r="A34" s="53"/>
+      <c r="A34" s="45"/>
       <c r="B34" s="10"/>
       <c r="C34" s="16">
         <v>3307</v>
@@ -1754,7 +1754,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="16">
-      <c r="A35" s="53"/>
+      <c r="A35" s="45"/>
       <c r="B35" s="10"/>
       <c r="C35" s="16">
         <v>3308</v>
@@ -1762,12 +1762,12 @@
       <c r="D35" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E35" s="44" t="s">
+      <c r="E35" s="36" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16">
-      <c r="A36" s="53"/>
+      <c r="A36" s="45"/>
       <c r="B36" s="10"/>
       <c r="C36" s="16">
         <v>3309</v>
@@ -1780,7 +1780,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="16">
-      <c r="A37" s="54"/>
+      <c r="A37" s="46"/>
       <c r="B37" s="18"/>
       <c r="C37" s="16">
         <v>3310</v>
@@ -1807,22 +1807,22 @@
       <c r="E39" s="1"/>
     </row>
     <row r="40" spans="1:5" ht="15.5">
-      <c r="A40" s="43" t="s">
+      <c r="A40" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="43"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="43"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="52"/>
+      <c r="D40" s="52"/>
+      <c r="E40" s="52"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="37" t="s">
+      <c r="C41" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="D41" s="37"/>
-      <c r="E41" s="37"/>
+      <c r="D41" s="47"/>
+      <c r="E41" s="47"/>
     </row>
     <row r="42" spans="1:5" ht="16.5" thickBot="1">
       <c r="A42" s="19" t="s">
@@ -1842,20 +1842,20 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="15">
-      <c r="A43" s="48" t="s">
+      <c r="A43" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B43" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C43" s="38" t="s">
+      <c r="C43" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="D43" s="38"/>
-      <c r="E43" s="39"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="50"/>
     </row>
     <row r="44" spans="1:5" ht="16">
-      <c r="A44" s="49"/>
+      <c r="A44" s="42"/>
       <c r="C44" s="11">
         <v>41002</v>
       </c>
@@ -1867,7 +1867,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="16">
-      <c r="A45" s="49"/>
+      <c r="A45" s="42"/>
       <c r="C45" s="11">
         <v>41003</v>
       </c>
@@ -1879,7 +1879,7 @@
       </c>
     </row>
     <row r="46" spans="1:5" ht="16">
-      <c r="A46" s="49"/>
+      <c r="A46" s="42"/>
       <c r="C46" s="11">
         <v>41004</v>
       </c>
@@ -1891,7 +1891,7 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="16">
-      <c r="A47" s="49"/>
+      <c r="A47" s="42"/>
       <c r="C47" s="11">
         <v>41005</v>
       </c>
@@ -1903,7 +1903,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="16">
-      <c r="A48" s="49"/>
+      <c r="A48" s="42"/>
       <c r="C48" s="11">
         <v>41111</v>
       </c>
@@ -1915,7 +1915,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" ht="16">
-      <c r="A49" s="49"/>
+      <c r="A49" s="42"/>
       <c r="C49" s="11">
         <v>41115</v>
       </c>
@@ -1927,7 +1927,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="16">
-      <c r="A50" s="49"/>
+      <c r="A50" s="42"/>
       <c r="C50" s="11">
         <v>41116</v>
       </c>
@@ -1939,7 +1939,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="16">
-      <c r="A51" s="49"/>
+      <c r="A51" s="42"/>
       <c r="C51" s="11">
         <v>41117</v>
       </c>
@@ -1951,15 +1951,15 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="49"/>
-      <c r="C52" s="37" t="s">
+      <c r="A52" s="42"/>
+      <c r="C52" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="D52" s="37"/>
-      <c r="E52" s="40"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="48"/>
     </row>
     <row r="53" spans="1:5" ht="16">
-      <c r="A53" s="49"/>
+      <c r="A53" s="42"/>
       <c r="C53" s="16">
         <v>42001</v>
       </c>
@@ -1971,7 +1971,7 @@
       </c>
     </row>
     <row r="54" spans="1:5" ht="16">
-      <c r="A54" s="49"/>
+      <c r="A54" s="42"/>
       <c r="C54" s="11">
         <v>42002</v>
       </c>
@@ -1983,7 +1983,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" ht="16">
-      <c r="A55" s="49"/>
+      <c r="A55" s="42"/>
       <c r="C55" s="11">
         <v>42003</v>
       </c>
@@ -1995,7 +1995,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="16">
-      <c r="A56" s="49"/>
+      <c r="A56" s="42"/>
       <c r="C56" s="11">
         <v>42004</v>
       </c>
@@ -2007,7 +2007,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" ht="16">
-      <c r="A57" s="49"/>
+      <c r="A57" s="42"/>
       <c r="C57" s="11">
         <v>42111</v>
       </c>
@@ -2019,7 +2019,7 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="16">
-      <c r="A58" s="49"/>
+      <c r="A58" s="42"/>
       <c r="C58" s="11">
         <v>42115</v>
       </c>
@@ -2031,7 +2031,7 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="16">
-      <c r="A59" s="49"/>
+      <c r="A59" s="42"/>
       <c r="C59" s="11">
         <v>42116</v>
       </c>
@@ -2043,7 +2043,7 @@
       </c>
     </row>
     <row r="60" spans="1:5" ht="16">
-      <c r="A60" s="49"/>
+      <c r="A60" s="42"/>
       <c r="C60" s="11">
         <v>42117</v>
       </c>
@@ -2055,15 +2055,15 @@
       </c>
     </row>
     <row r="61" spans="1:5">
-      <c r="A61" s="49"/>
-      <c r="C61" s="37" t="s">
+      <c r="A61" s="42"/>
+      <c r="C61" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="D61" s="37"/>
-      <c r="E61" s="40"/>
+      <c r="D61" s="47"/>
+      <c r="E61" s="48"/>
     </row>
     <row r="62" spans="1:5" ht="16">
-      <c r="A62" s="49"/>
+      <c r="A62" s="42"/>
       <c r="C62" s="16">
         <v>43001</v>
       </c>
@@ -2075,7 +2075,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" ht="16">
-      <c r="A63" s="49"/>
+      <c r="A63" s="42"/>
       <c r="C63" s="11">
         <v>43002</v>
       </c>
@@ -2087,7 +2087,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="16">
-      <c r="A64" s="49"/>
+      <c r="A64" s="42"/>
       <c r="C64" s="16">
         <v>43003</v>
       </c>
@@ -2099,7 +2099,7 @@
       </c>
     </row>
     <row r="65" spans="1:5" ht="16">
-      <c r="A65" s="49"/>
+      <c r="A65" s="42"/>
       <c r="C65" s="11">
         <v>43004</v>
       </c>
@@ -2111,7 +2111,7 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="16">
-      <c r="A66" s="49"/>
+      <c r="A66" s="42"/>
       <c r="C66" s="11">
         <v>43111</v>
       </c>
@@ -2123,7 +2123,7 @@
       </c>
     </row>
     <row r="67" spans="1:5" ht="16">
-      <c r="A67" s="49"/>
+      <c r="A67" s="42"/>
       <c r="C67" s="11">
         <v>43115</v>
       </c>
@@ -2135,7 +2135,7 @@
       </c>
     </row>
     <row r="68" spans="1:5" ht="16">
-      <c r="A68" s="49"/>
+      <c r="A68" s="42"/>
       <c r="C68" s="11">
         <v>43116</v>
       </c>
@@ -2147,7 +2147,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" ht="16.5" thickBot="1">
-      <c r="A69" s="50"/>
+      <c r="A69" s="43"/>
       <c r="C69" s="12">
         <v>43117</v>
       </c>
@@ -2159,20 +2159,20 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="15">
-      <c r="A70" s="48" t="s">
+      <c r="A70" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B70" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C70" s="38" t="s">
+      <c r="C70" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="D70" s="38"/>
-      <c r="E70" s="39"/>
+      <c r="D70" s="49"/>
+      <c r="E70" s="50"/>
     </row>
     <row r="71" spans="1:5" ht="16">
-      <c r="A71" s="49"/>
+      <c r="A71" s="42"/>
       <c r="B71" s="23"/>
       <c r="C71" s="11">
         <v>41002</v>
@@ -2185,7 +2185,7 @@
       </c>
     </row>
     <row r="72" spans="1:5" ht="16">
-      <c r="A72" s="49"/>
+      <c r="A72" s="42"/>
       <c r="B72" s="23"/>
       <c r="C72" s="11">
         <v>41003</v>
@@ -2198,7 +2198,7 @@
       </c>
     </row>
     <row r="73" spans="1:5" ht="16">
-      <c r="A73" s="49"/>
+      <c r="A73" s="42"/>
       <c r="B73" s="23"/>
       <c r="C73" s="11">
         <v>41004</v>
@@ -2211,7 +2211,7 @@
       </c>
     </row>
     <row r="74" spans="1:5" ht="16">
-      <c r="A74" s="49"/>
+      <c r="A74" s="42"/>
       <c r="B74" s="23"/>
       <c r="C74" s="11">
         <v>41005</v>
@@ -2224,7 +2224,7 @@
       </c>
     </row>
     <row r="75" spans="1:5" ht="16">
-      <c r="A75" s="49"/>
+      <c r="A75" s="42"/>
       <c r="B75" s="23"/>
       <c r="C75" s="11">
         <v>41101</v>
@@ -2237,7 +2237,7 @@
       </c>
     </row>
     <row r="76" spans="1:5" ht="16">
-      <c r="A76" s="49"/>
+      <c r="A76" s="42"/>
       <c r="B76" s="23"/>
       <c r="C76" s="11">
         <v>41102</v>
@@ -2250,7 +2250,7 @@
       </c>
     </row>
     <row r="77" spans="1:5" ht="16">
-      <c r="A77" s="49"/>
+      <c r="A77" s="42"/>
       <c r="B77" s="23"/>
       <c r="C77" s="11">
         <v>41131</v>
@@ -2258,12 +2258,12 @@
       <c r="D77" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E77" s="45" t="s">
+      <c r="E77" s="37" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="16">
-      <c r="A78" s="49"/>
+      <c r="A78" s="42"/>
       <c r="B78" s="23"/>
       <c r="C78" s="11">
         <v>41135</v>
@@ -2271,21 +2271,21 @@
       <c r="D78" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E78" s="45" t="s">
+      <c r="E78" s="37" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15">
-      <c r="A79" s="49"/>
+      <c r="A79" s="42"/>
       <c r="B79" s="23"/>
-      <c r="C79" s="37" t="s">
+      <c r="C79" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="D79" s="37"/>
-      <c r="E79" s="40"/>
+      <c r="D79" s="47"/>
+      <c r="E79" s="48"/>
     </row>
     <row r="80" spans="1:5" ht="16">
-      <c r="A80" s="49"/>
+      <c r="A80" s="42"/>
       <c r="B80" s="23"/>
       <c r="C80" s="4" t="s">
         <v>3</v>
@@ -2298,7 +2298,7 @@
       </c>
     </row>
     <row r="81" spans="1:5" ht="16">
-      <c r="A81" s="49"/>
+      <c r="A81" s="42"/>
       <c r="B81" s="23"/>
       <c r="C81" s="16">
         <v>42001</v>
@@ -2311,7 +2311,7 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="16">
-      <c r="A82" s="49"/>
+      <c r="A82" s="42"/>
       <c r="B82" s="23"/>
       <c r="C82" s="11">
         <v>42002</v>
@@ -2324,7 +2324,7 @@
       </c>
     </row>
     <row r="83" spans="1:5" ht="16">
-      <c r="A83" s="49"/>
+      <c r="A83" s="42"/>
       <c r="B83" s="23"/>
       <c r="C83" s="11">
         <v>42003</v>
@@ -2337,7 +2337,7 @@
       </c>
     </row>
     <row r="84" spans="1:5" ht="16">
-      <c r="A84" s="49"/>
+      <c r="A84" s="42"/>
       <c r="B84" s="23"/>
       <c r="C84" s="11">
         <v>42004</v>
@@ -2350,7 +2350,7 @@
       </c>
     </row>
     <row r="85" spans="1:5" ht="16">
-      <c r="A85" s="49"/>
+      <c r="A85" s="42"/>
       <c r="B85" s="23"/>
       <c r="C85" s="11">
         <v>42101</v>
@@ -2363,7 +2363,7 @@
       </c>
     </row>
     <row r="86" spans="1:5" ht="16">
-      <c r="A86" s="49"/>
+      <c r="A86" s="42"/>
       <c r="B86" s="23"/>
       <c r="C86" s="11">
         <v>42102</v>
@@ -2376,7 +2376,7 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="16">
-      <c r="A87" s="49"/>
+      <c r="A87" s="42"/>
       <c r="B87" s="23"/>
       <c r="C87" s="11">
         <v>42131</v>
@@ -2384,12 +2384,12 @@
       <c r="D87" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E87" s="45" t="s">
+      <c r="E87" s="37" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="16">
-      <c r="A88" s="49"/>
+      <c r="A88" s="42"/>
       <c r="B88" s="23"/>
       <c r="C88" s="11">
         <v>42135</v>
@@ -2397,20 +2397,20 @@
       <c r="D88" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="E88" s="45" t="s">
+      <c r="E88" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="89" spans="1:5">
-      <c r="A89" s="49"/>
-      <c r="C89" s="37" t="s">
+      <c r="A89" s="42"/>
+      <c r="C89" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="D89" s="37"/>
-      <c r="E89" s="40"/>
+      <c r="D89" s="47"/>
+      <c r="E89" s="48"/>
     </row>
     <row r="90" spans="1:5" ht="16">
-      <c r="A90" s="49"/>
+      <c r="A90" s="42"/>
       <c r="C90" s="16">
         <v>43001</v>
       </c>
@@ -2422,7 +2422,7 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="16">
-      <c r="A91" s="49"/>
+      <c r="A91" s="42"/>
       <c r="C91" s="11">
         <v>43002</v>
       </c>
@@ -2434,7 +2434,7 @@
       </c>
     </row>
     <row r="92" spans="1:5" ht="16">
-      <c r="A92" s="49"/>
+      <c r="A92" s="42"/>
       <c r="C92" s="16">
         <v>43003</v>
       </c>
@@ -2446,11 +2446,11 @@
       </c>
     </row>
     <row r="93" spans="1:5" ht="16">
-      <c r="A93" s="49"/>
+      <c r="A93" s="42"/>
       <c r="C93" s="11">
         <v>43004</v>
       </c>
-      <c r="D93" s="44" t="s">
+      <c r="D93" s="36" t="s">
         <v>84</v>
       </c>
       <c r="E93" s="27" t="s">
@@ -2458,11 +2458,11 @@
       </c>
     </row>
     <row r="94" spans="1:5" ht="16">
-      <c r="A94" s="49"/>
+      <c r="A94" s="42"/>
       <c r="C94" s="11">
         <v>43101</v>
       </c>
-      <c r="D94" s="44" t="s">
+      <c r="D94" s="36" t="s">
         <v>83</v>
       </c>
       <c r="E94" s="27" t="s">
@@ -2470,11 +2470,11 @@
       </c>
     </row>
     <row r="95" spans="1:5" ht="16">
-      <c r="A95" s="49"/>
+      <c r="A95" s="42"/>
       <c r="C95" s="11">
         <v>43102</v>
       </c>
-      <c r="D95" s="44" t="s">
+      <c r="D95" s="36" t="s">
         <v>82</v>
       </c>
       <c r="E95" s="27" t="s">
@@ -2482,11 +2482,11 @@
       </c>
     </row>
     <row r="96" spans="1:5" ht="16.5" thickBot="1">
-      <c r="A96" s="50"/>
+      <c r="A96" s="43"/>
       <c r="C96" s="11">
         <v>43131</v>
       </c>
-      <c r="D96" s="44" t="s">
+      <c r="D96" s="36" t="s">
         <v>81</v>
       </c>
       <c r="E96" s="27" t="s">
@@ -2498,7 +2498,7 @@
       <c r="C97" s="12">
         <v>43135</v>
       </c>
-      <c r="D97" s="46" t="s">
+      <c r="D97" s="38" t="s">
         <v>80</v>
       </c>
       <c r="E97" s="25" t="s">
@@ -2506,20 +2506,20 @@
       </c>
     </row>
     <row r="98" spans="1:5" ht="15">
-      <c r="A98" s="48" t="s">
+      <c r="A98" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B98" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C98" s="38" t="s">
+      <c r="C98" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="D98" s="38"/>
-      <c r="E98" s="39"/>
+      <c r="D98" s="49"/>
+      <c r="E98" s="50"/>
     </row>
     <row r="99" spans="1:5" ht="16">
-      <c r="A99" s="49"/>
+      <c r="A99" s="42"/>
       <c r="B99" s="23"/>
       <c r="C99" s="11">
         <v>41002</v>
@@ -2532,7 +2532,7 @@
       </c>
     </row>
     <row r="100" spans="1:5" ht="16">
-      <c r="A100" s="49"/>
+      <c r="A100" s="42"/>
       <c r="B100" s="23"/>
       <c r="C100" s="11">
         <v>41003</v>
@@ -2545,7 +2545,7 @@
       </c>
     </row>
     <row r="101" spans="1:5" ht="16">
-      <c r="A101" s="49"/>
+      <c r="A101" s="42"/>
       <c r="B101" s="23"/>
       <c r="C101" s="11">
         <v>41004</v>
@@ -2558,7 +2558,7 @@
       </c>
     </row>
     <row r="102" spans="1:5" ht="16">
-      <c r="A102" s="49"/>
+      <c r="A102" s="42"/>
       <c r="B102" s="23"/>
       <c r="C102" s="11">
         <v>41005</v>
@@ -2571,7 +2571,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" ht="16">
-      <c r="A103" s="49"/>
+      <c r="A103" s="42"/>
       <c r="B103" s="23"/>
       <c r="C103" s="11">
         <v>41101</v>
@@ -2584,7 +2584,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" ht="16">
-      <c r="A104" s="49"/>
+      <c r="A104" s="42"/>
       <c r="B104" s="23"/>
       <c r="C104" s="11">
         <v>41102</v>
@@ -2597,7 +2597,7 @@
       </c>
     </row>
     <row r="105" spans="1:5" ht="16">
-      <c r="A105" s="49"/>
+      <c r="A105" s="42"/>
       <c r="B105" s="23"/>
       <c r="C105" s="11">
         <v>41191</v>
@@ -2610,7 +2610,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" ht="16">
-      <c r="A106" s="49"/>
+      <c r="A106" s="42"/>
       <c r="B106" s="23"/>
       <c r="C106" s="11">
         <v>41195</v>
@@ -2623,16 +2623,16 @@
       </c>
     </row>
     <row r="107" spans="1:5" ht="15">
-      <c r="A107" s="49"/>
+      <c r="A107" s="42"/>
       <c r="B107" s="23"/>
-      <c r="C107" s="37" t="s">
+      <c r="C107" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="D107" s="37"/>
-      <c r="E107" s="40"/>
+      <c r="D107" s="47"/>
+      <c r="E107" s="48"/>
     </row>
     <row r="108" spans="1:5" ht="16">
-      <c r="A108" s="49"/>
+      <c r="A108" s="42"/>
       <c r="B108" s="23"/>
       <c r="C108" s="4" t="s">
         <v>3</v>
@@ -2645,7 +2645,7 @@
       </c>
     </row>
     <row r="109" spans="1:5" ht="16">
-      <c r="A109" s="49"/>
+      <c r="A109" s="42"/>
       <c r="B109" s="23"/>
       <c r="C109" s="16">
         <v>42001</v>
@@ -2658,7 +2658,7 @@
       </c>
     </row>
     <row r="110" spans="1:5" ht="16">
-      <c r="A110" s="49"/>
+      <c r="A110" s="42"/>
       <c r="B110" s="23"/>
       <c r="C110" s="11">
         <v>42002</v>
@@ -2671,7 +2671,7 @@
       </c>
     </row>
     <row r="111" spans="1:5" ht="16">
-      <c r="A111" s="49"/>
+      <c r="A111" s="42"/>
       <c r="B111" s="23"/>
       <c r="C111" s="11">
         <v>42003</v>
@@ -2684,7 +2684,7 @@
       </c>
     </row>
     <row r="112" spans="1:5" ht="16">
-      <c r="A112" s="49"/>
+      <c r="A112" s="42"/>
       <c r="B112" s="23"/>
       <c r="C112" s="11">
         <v>42004</v>
@@ -2697,7 +2697,7 @@
       </c>
     </row>
     <row r="113" spans="1:5" ht="16">
-      <c r="A113" s="49"/>
+      <c r="A113" s="42"/>
       <c r="B113" s="23"/>
       <c r="C113" s="11">
         <v>42101</v>
@@ -2710,7 +2710,7 @@
       </c>
     </row>
     <row r="114" spans="1:5" ht="16">
-      <c r="A114" s="49"/>
+      <c r="A114" s="42"/>
       <c r="B114" s="23"/>
       <c r="C114" s="11">
         <v>42102</v>
@@ -2723,12 +2723,12 @@
       </c>
     </row>
     <row r="115" spans="1:5" ht="16">
-      <c r="A115" s="49"/>
+      <c r="A115" s="42"/>
       <c r="B115" s="23"/>
       <c r="C115" s="11">
         <v>42191</v>
       </c>
-      <c r="D115" s="44" t="s">
+      <c r="D115" s="36" t="s">
         <v>85</v>
       </c>
       <c r="E115" s="27" t="s">
@@ -2736,12 +2736,12 @@
       </c>
     </row>
     <row r="116" spans="1:5" ht="16">
-      <c r="A116" s="49"/>
+      <c r="A116" s="42"/>
       <c r="B116" s="23"/>
       <c r="C116" s="11">
         <v>42195</v>
       </c>
-      <c r="D116" s="44" t="s">
+      <c r="D116" s="36" t="s">
         <v>86</v>
       </c>
       <c r="E116" s="27" t="s">
@@ -2749,15 +2749,15 @@
       </c>
     </row>
     <row r="117" spans="1:5">
-      <c r="A117" s="49"/>
-      <c r="C117" s="37" t="s">
+      <c r="A117" s="42"/>
+      <c r="C117" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="D117" s="37"/>
-      <c r="E117" s="40"/>
+      <c r="D117" s="47"/>
+      <c r="E117" s="48"/>
     </row>
     <row r="118" spans="1:5" ht="16">
-      <c r="A118" s="49"/>
+      <c r="A118" s="42"/>
       <c r="C118" s="16">
         <v>43001</v>
       </c>
@@ -2769,7 +2769,7 @@
       </c>
     </row>
     <row r="119" spans="1:5" ht="16">
-      <c r="A119" s="49"/>
+      <c r="A119" s="42"/>
       <c r="C119" s="11">
         <v>43002</v>
       </c>
@@ -2781,7 +2781,7 @@
       </c>
     </row>
     <row r="120" spans="1:5" ht="16">
-      <c r="A120" s="49"/>
+      <c r="A120" s="42"/>
       <c r="C120" s="16">
         <v>43003</v>
       </c>
@@ -2793,11 +2793,11 @@
       </c>
     </row>
     <row r="121" spans="1:5" ht="16">
-      <c r="A121" s="49"/>
+      <c r="A121" s="42"/>
       <c r="C121" s="11">
         <v>43004</v>
       </c>
-      <c r="D121" s="44" t="s">
+      <c r="D121" s="36" t="s">
         <v>84</v>
       </c>
       <c r="E121" s="27" t="s">
@@ -2805,11 +2805,11 @@
       </c>
     </row>
     <row r="122" spans="1:5" ht="16">
-      <c r="A122" s="49"/>
+      <c r="A122" s="42"/>
       <c r="C122" s="11">
         <v>43101</v>
       </c>
-      <c r="D122" s="44" t="s">
+      <c r="D122" s="36" t="s">
         <v>83</v>
       </c>
       <c r="E122" s="27" t="s">
@@ -2817,11 +2817,11 @@
       </c>
     </row>
     <row r="123" spans="1:5" ht="16">
-      <c r="A123" s="49"/>
+      <c r="A123" s="42"/>
       <c r="C123" s="11">
         <v>43102</v>
       </c>
-      <c r="D123" s="44" t="s">
+      <c r="D123" s="36" t="s">
         <v>82</v>
       </c>
       <c r="E123" s="27" t="s">
@@ -2829,11 +2829,11 @@
       </c>
     </row>
     <row r="124" spans="1:5" ht="16.5" thickBot="1">
-      <c r="A124" s="50"/>
+      <c r="A124" s="43"/>
       <c r="C124" s="11">
         <v>43191</v>
       </c>
-      <c r="D124" s="44" t="s">
+      <c r="D124" s="36" t="s">
         <v>87</v>
       </c>
       <c r="E124" s="27" t="s">
@@ -2846,7 +2846,7 @@
       <c r="C125" s="32">
         <v>43195</v>
       </c>
-      <c r="D125" s="47" t="s">
+      <c r="D125" s="39" t="s">
         <v>88</v>
       </c>
       <c r="E125" s="33" t="s">
@@ -2854,20 +2854,20 @@
       </c>
     </row>
     <row r="126" spans="1:5" ht="15">
-      <c r="A126" s="48" t="s">
+      <c r="A126" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B126" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C126" s="38" t="s">
+      <c r="C126" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="D126" s="38"/>
-      <c r="E126" s="39"/>
+      <c r="D126" s="49"/>
+      <c r="E126" s="50"/>
     </row>
     <row r="127" spans="1:5" ht="16">
-      <c r="A127" s="49"/>
+      <c r="A127" s="42"/>
       <c r="B127" s="23"/>
       <c r="C127" s="11">
         <v>41002</v>
@@ -2880,7 +2880,7 @@
       </c>
     </row>
     <row r="128" spans="1:5" ht="16">
-      <c r="A128" s="49"/>
+      <c r="A128" s="42"/>
       <c r="B128" s="23"/>
       <c r="C128" s="11">
         <v>41003</v>
@@ -2893,7 +2893,7 @@
       </c>
     </row>
     <row r="129" spans="1:5" ht="16">
-      <c r="A129" s="49"/>
+      <c r="A129" s="42"/>
       <c r="B129" s="23"/>
       <c r="C129" s="11">
         <v>41004</v>
@@ -2906,7 +2906,7 @@
       </c>
     </row>
     <row r="130" spans="1:5" ht="16">
-      <c r="A130" s="49"/>
+      <c r="A130" s="42"/>
       <c r="B130" s="23"/>
       <c r="C130" s="11">
         <v>41005</v>
@@ -2919,7 +2919,7 @@
       </c>
     </row>
     <row r="131" spans="1:5" ht="16">
-      <c r="A131" s="49"/>
+      <c r="A131" s="42"/>
       <c r="B131" s="23"/>
       <c r="C131" s="11">
         <v>41091</v>
@@ -2932,12 +2932,12 @@
       </c>
     </row>
     <row r="132" spans="1:5" ht="16">
-      <c r="A132" s="49"/>
+      <c r="A132" s="42"/>
       <c r="B132" s="23"/>
       <c r="C132" s="11">
         <v>41095</v>
       </c>
-      <c r="D132" s="44" t="s">
+      <c r="D132" s="36" t="s">
         <v>89</v>
       </c>
       <c r="E132" s="27" t="s">
@@ -2945,7 +2945,7 @@
       </c>
     </row>
     <row r="133" spans="1:5" ht="16">
-      <c r="A133" s="49"/>
+      <c r="A133" s="42"/>
       <c r="B133" s="23"/>
       <c r="C133" s="11">
         <v>41191</v>
@@ -2958,7 +2958,7 @@
       </c>
     </row>
     <row r="134" spans="1:5" ht="16">
-      <c r="A134" s="49"/>
+      <c r="A134" s="42"/>
       <c r="B134" s="23"/>
       <c r="C134" s="11">
         <v>41195</v>
@@ -2971,16 +2971,16 @@
       </c>
     </row>
     <row r="135" spans="1:5" ht="15">
-      <c r="A135" s="49"/>
+      <c r="A135" s="42"/>
       <c r="B135" s="23"/>
-      <c r="C135" s="37" t="s">
+      <c r="C135" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="D135" s="37"/>
-      <c r="E135" s="40"/>
+      <c r="D135" s="47"/>
+      <c r="E135" s="48"/>
     </row>
     <row r="136" spans="1:5" ht="16">
-      <c r="A136" s="49"/>
+      <c r="A136" s="42"/>
       <c r="B136" s="23"/>
       <c r="C136" s="4" t="s">
         <v>3</v>
@@ -2993,7 +2993,7 @@
       </c>
     </row>
     <row r="137" spans="1:5" ht="16">
-      <c r="A137" s="49"/>
+      <c r="A137" s="42"/>
       <c r="B137" s="23"/>
       <c r="C137" s="16">
         <v>42001</v>
@@ -3006,7 +3006,7 @@
       </c>
     </row>
     <row r="138" spans="1:5" ht="16">
-      <c r="A138" s="49"/>
+      <c r="A138" s="42"/>
       <c r="B138" s="23"/>
       <c r="C138" s="11">
         <v>42002</v>
@@ -3019,7 +3019,7 @@
       </c>
     </row>
     <row r="139" spans="1:5" ht="16">
-      <c r="A139" s="49"/>
+      <c r="A139" s="42"/>
       <c r="B139" s="23"/>
       <c r="C139" s="11">
         <v>42003</v>
@@ -3032,7 +3032,7 @@
       </c>
     </row>
     <row r="140" spans="1:5" ht="16">
-      <c r="A140" s="49"/>
+      <c r="A140" s="42"/>
       <c r="B140" s="23"/>
       <c r="C140" s="11">
         <v>42004</v>
@@ -3045,7 +3045,7 @@
       </c>
     </row>
     <row r="141" spans="1:5" ht="16">
-      <c r="A141" s="49"/>
+      <c r="A141" s="42"/>
       <c r="B141" s="23"/>
       <c r="C141" s="11">
         <v>42091</v>
@@ -3058,12 +3058,12 @@
       </c>
     </row>
     <row r="142" spans="1:5" ht="16">
-      <c r="A142" s="49"/>
+      <c r="A142" s="42"/>
       <c r="B142" s="23"/>
       <c r="C142" s="11">
         <v>42095</v>
       </c>
-      <c r="D142" s="44" t="s">
+      <c r="D142" s="36" t="s">
         <v>91</v>
       </c>
       <c r="E142" s="27" t="s">
@@ -3071,12 +3071,12 @@
       </c>
     </row>
     <row r="143" spans="1:5" ht="16">
-      <c r="A143" s="49"/>
+      <c r="A143" s="42"/>
       <c r="B143" s="23"/>
       <c r="C143" s="11">
         <v>42191</v>
       </c>
-      <c r="D143" s="44" t="s">
+      <c r="D143" s="36" t="s">
         <v>85</v>
       </c>
       <c r="E143" s="27" t="s">
@@ -3084,12 +3084,12 @@
       </c>
     </row>
     <row r="144" spans="1:5" ht="16">
-      <c r="A144" s="49"/>
+      <c r="A144" s="42"/>
       <c r="B144" s="23"/>
       <c r="C144" s="11">
         <v>42195</v>
       </c>
-      <c r="D144" s="44" t="s">
+      <c r="D144" s="36" t="s">
         <v>86</v>
       </c>
       <c r="E144" s="27" t="s">
@@ -3097,15 +3097,15 @@
       </c>
     </row>
     <row r="145" spans="1:5">
-      <c r="A145" s="49"/>
-      <c r="C145" s="37" t="s">
+      <c r="A145" s="42"/>
+      <c r="C145" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="D145" s="37"/>
-      <c r="E145" s="40"/>
+      <c r="D145" s="47"/>
+      <c r="E145" s="48"/>
     </row>
     <row r="146" spans="1:5" ht="16">
-      <c r="A146" s="49"/>
+      <c r="A146" s="42"/>
       <c r="C146" s="16">
         <v>43001</v>
       </c>
@@ -3117,7 +3117,7 @@
       </c>
     </row>
     <row r="147" spans="1:5" ht="16">
-      <c r="A147" s="49"/>
+      <c r="A147" s="42"/>
       <c r="C147" s="11">
         <v>43002</v>
       </c>
@@ -3129,7 +3129,7 @@
       </c>
     </row>
     <row r="148" spans="1:5" ht="16">
-      <c r="A148" s="49"/>
+      <c r="A148" s="42"/>
       <c r="C148" s="16">
         <v>43003</v>
       </c>
@@ -3141,11 +3141,11 @@
       </c>
     </row>
     <row r="149" spans="1:5" ht="16">
-      <c r="A149" s="49"/>
+      <c r="A149" s="42"/>
       <c r="C149" s="11">
         <v>43004</v>
       </c>
-      <c r="D149" s="44" t="s">
+      <c r="D149" s="36" t="s">
         <v>90</v>
       </c>
       <c r="E149" s="27" t="s">
@@ -3153,11 +3153,11 @@
       </c>
     </row>
     <row r="150" spans="1:5" ht="16">
-      <c r="A150" s="49"/>
+      <c r="A150" s="42"/>
       <c r="C150" s="11">
         <v>43091</v>
       </c>
-      <c r="D150" s="44" t="s">
+      <c r="D150" s="36" t="s">
         <v>92</v>
       </c>
       <c r="E150" s="27" t="s">
@@ -3165,11 +3165,11 @@
       </c>
     </row>
     <row r="151" spans="1:5" ht="16">
-      <c r="A151" s="49"/>
+      <c r="A151" s="42"/>
       <c r="C151" s="11">
         <v>43095</v>
       </c>
-      <c r="D151" s="44" t="s">
+      <c r="D151" s="36" t="s">
         <v>91</v>
       </c>
       <c r="E151" s="27" t="s">
@@ -3177,11 +3177,11 @@
       </c>
     </row>
     <row r="152" spans="1:5" ht="16.5" thickBot="1">
-      <c r="A152" s="50"/>
+      <c r="A152" s="43"/>
       <c r="C152" s="11">
         <v>43191</v>
       </c>
-      <c r="D152" s="44" t="s">
+      <c r="D152" s="36" t="s">
         <v>85</v>
       </c>
       <c r="E152" s="27" t="s">
@@ -3194,7 +3194,7 @@
       <c r="C153" s="32">
         <v>43195</v>
       </c>
-      <c r="D153" s="47" t="s">
+      <c r="D153" s="39" t="s">
         <v>86</v>
       </c>
       <c r="E153" s="33" t="s">
@@ -3329,21 +3329,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A43:A69"/>
-    <mergeCell ref="A70:A96"/>
-    <mergeCell ref="A98:A124"/>
-    <mergeCell ref="A126:A152"/>
-    <mergeCell ref="A5:A37"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="C117:E117"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="C145:E145"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="C98:E98"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C52:E52"/>
@@ -3353,6 +3338,21 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="C117:E117"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="C145:E145"/>
+    <mergeCell ref="A43:A69"/>
+    <mergeCell ref="A70:A96"/>
+    <mergeCell ref="A98:A124"/>
+    <mergeCell ref="A126:A152"/>
+    <mergeCell ref="A5:A37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>